<commit_message>
add all ghg scenarios, new policy files, configs, update figures etc
</commit_message>
<xml_diff>
--- a/analysis/query/iamc_format/msg_gcam_comparison_all.xlsx
+++ b/analysis/query/iamc_format/msg_gcam_comparison_all.xlsx
@@ -488,22 +488,22 @@
         </is>
       </c>
       <c r="F3">
-        <v>119.86</v>
+        <v>116.8</v>
       </c>
       <c r="G3">
-        <v>156.72</v>
+        <v>137.64</v>
       </c>
       <c r="H3">
-        <v>201.27</v>
+        <v>166.84</v>
       </c>
       <c r="I3">
-        <v>279.15</v>
+        <v>224.75</v>
       </c>
       <c r="J3">
-        <v>380.73</v>
+        <v>303.5</v>
       </c>
       <c r="K3">
-        <v>479.02</v>
+        <v>377.59</v>
       </c>
     </row>
     <row r="4">
@@ -533,22 +533,22 @@
         </is>
       </c>
       <c r="F4">
-        <v>45.57</v>
+        <v>42.5</v>
       </c>
       <c r="G4">
-        <v>-67.36</v>
+        <v>-86.44</v>
       </c>
       <c r="H4">
-        <v>-181.37</v>
+        <v>-215.8</v>
       </c>
       <c r="I4">
-        <v>-286.52</v>
+        <v>-340.91</v>
       </c>
       <c r="J4">
-        <v>-394.33</v>
+        <v>-471.56</v>
       </c>
       <c r="K4">
-        <v>-577.36</v>
+        <v>-678.79</v>
       </c>
     </row>
     <row r="5">
@@ -578,26 +578,26 @@
         </is>
       </c>
       <c r="F5">
-        <v>61.3</v>
+        <v>57.2</v>
       </c>
       <c r="G5">
-        <v>-30.1</v>
+        <v>-38.6</v>
       </c>
       <c r="H5">
-        <v>-47.4</v>
+        <v>-56.4</v>
       </c>
       <c r="I5">
-        <v>-50.7</v>
+        <v>-60.3</v>
       </c>
       <c r="J5">
-        <v>-50.9</v>
+        <v>-60.8</v>
       </c>
       <c r="K5">
-        <v>-54.7</v>
+        <v>-64.3</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>MSG 2.2x higher at 2050</t>
+          <t>MSG 2.8x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="F7">
-        <v>205.73</v>
+        <v>199.72</v>
       </c>
       <c r="G7">
-        <v>251.47</v>
+        <v>224.83</v>
       </c>
       <c r="H7">
-        <v>295.55</v>
+        <v>251.69</v>
       </c>
       <c r="I7">
-        <v>368.24</v>
+        <v>304.51</v>
       </c>
       <c r="J7">
-        <v>464.01</v>
+        <v>378.34</v>
       </c>
       <c r="K7">
-        <v>547.65</v>
+        <v>441.49</v>
       </c>
     </row>
     <row r="8">
@@ -718,22 +718,22 @@
         </is>
       </c>
       <c r="F8">
-        <v>54.53</v>
+        <v>48.52</v>
       </c>
       <c r="G8">
-        <v>34.94</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H8">
-        <v>-110.33</v>
+        <v>-154.19</v>
       </c>
       <c r="I8">
-        <v>-219.47</v>
+        <v>-283.2</v>
       </c>
       <c r="J8">
-        <v>-355.78</v>
+        <v>-441.44</v>
       </c>
       <c r="K8">
-        <v>-568.33</v>
+        <v>-674.49</v>
       </c>
     </row>
     <row r="9">
@@ -763,26 +763,26 @@
         </is>
       </c>
       <c r="F9">
-        <v>36.1</v>
+        <v>32.1</v>
       </c>
       <c r="G9">
-        <v>16.1</v>
+        <v>3.8</v>
       </c>
       <c r="H9">
-        <v>-27.2</v>
+        <v>-38</v>
       </c>
       <c r="I9">
-        <v>-37.3</v>
+        <v>-48.2</v>
       </c>
       <c r="J9">
-        <v>-43.4</v>
+        <v>-53.8</v>
       </c>
       <c r="K9">
-        <v>-50.9</v>
+        <v>-60.4</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>MSG 2.0x higher at 2050</t>
+          <t>MSG 2.5x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -858,22 +858,22 @@
         </is>
       </c>
       <c r="F11">
-        <v>57.74</v>
+        <v>54.14</v>
       </c>
       <c r="G11">
-        <v>74.5</v>
+        <v>66.69</v>
       </c>
       <c r="H11">
-        <v>95.66</v>
+        <v>82.91</v>
       </c>
       <c r="I11">
-        <v>138.53</v>
+        <v>117.19</v>
       </c>
       <c r="J11">
-        <v>189.22</v>
+        <v>160.84</v>
       </c>
       <c r="K11">
-        <v>225.29</v>
+        <v>193.73</v>
       </c>
     </row>
     <row r="12">
@@ -903,22 +903,22 @@
         </is>
       </c>
       <c r="F12">
-        <v>47.82</v>
+        <v>44.22</v>
       </c>
       <c r="G12">
-        <v>-104.53</v>
+        <v>-112.34</v>
       </c>
       <c r="H12">
-        <v>-107.87</v>
+        <v>-120.63</v>
       </c>
       <c r="I12">
-        <v>-92.05</v>
+        <v>-113.4</v>
       </c>
       <c r="J12">
-        <v>-48.5</v>
+        <v>-76.89</v>
       </c>
       <c r="K12">
-        <v>32.08</v>
+        <v>0.52</v>
       </c>
     </row>
     <row r="13">
@@ -948,26 +948,26 @@
         </is>
       </c>
       <c r="F13">
-        <v>482.1</v>
+        <v>445.9</v>
       </c>
       <c r="G13">
-        <v>-58.4</v>
+        <v>-62.8</v>
       </c>
       <c r="H13">
-        <v>-53</v>
+        <v>-59.3</v>
       </c>
       <c r="I13">
-        <v>-39.9</v>
+        <v>-49.2</v>
       </c>
       <c r="J13">
-        <v>-20.4</v>
+        <v>-32.3</v>
       </c>
       <c r="K13">
-        <v>16.6</v>
+        <v>0.3</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>GCAM 1.2x higher at 2050</t>
+          <t>~0% gap at 2050</t>
         </is>
       </c>
     </row>
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="F15">
-        <v>63.93</v>
+        <v>62.2</v>
       </c>
       <c r="G15">
-        <v>81.15000000000001</v>
+        <v>71.79000000000001</v>
       </c>
       <c r="H15">
-        <v>96.61</v>
+        <v>81.48999999999999</v>
       </c>
       <c r="I15">
-        <v>119.99</v>
+        <v>98.31999999999999</v>
       </c>
       <c r="J15">
-        <v>145.8</v>
+        <v>117.59</v>
       </c>
       <c r="K15">
-        <v>165.65</v>
+        <v>131.58</v>
       </c>
     </row>
     <row r="16">
@@ -1088,22 +1088,22 @@
         </is>
       </c>
       <c r="F16">
-        <v>-19.84</v>
+        <v>-21.58</v>
       </c>
       <c r="G16">
-        <v>-4.69</v>
+        <v>-14.06</v>
       </c>
       <c r="H16">
-        <v>-15.82</v>
+        <v>-30.95</v>
       </c>
       <c r="I16">
-        <v>7.55</v>
+        <v>-14.12</v>
       </c>
       <c r="J16">
-        <v>33.37</v>
+        <v>5.15</v>
       </c>
       <c r="K16">
-        <v>53.22</v>
+        <v>19.14</v>
       </c>
     </row>
     <row r="17">
@@ -1133,26 +1133,26 @@
         </is>
       </c>
       <c r="F17">
-        <v>-23.7</v>
+        <v>-25.8</v>
       </c>
       <c r="G17">
-        <v>-5.5</v>
+        <v>-16.4</v>
       </c>
       <c r="H17">
-        <v>-14.1</v>
+        <v>-27.5</v>
       </c>
       <c r="I17">
-        <v>6.7</v>
+        <v>-12.6</v>
       </c>
       <c r="J17">
-        <v>29.7</v>
+        <v>4.6</v>
       </c>
       <c r="K17">
-        <v>47.3</v>
+        <v>17</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>GCAM 1.5x higher at 2050</t>
+          <t>GCAM 1.2x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -1413,22 +1413,22 @@
         </is>
       </c>
       <c r="F23">
-        <v>54.79</v>
+        <v>87.11</v>
       </c>
       <c r="G23">
-        <v>212.4</v>
+        <v>273.64</v>
       </c>
       <c r="H23">
-        <v>381.45</v>
+        <v>464.79</v>
       </c>
       <c r="I23">
-        <v>620.04</v>
+        <v>741.9400000000001</v>
       </c>
       <c r="J23">
-        <v>898.62</v>
+        <v>1076.56</v>
       </c>
       <c r="K23">
-        <v>1151.62</v>
+        <v>1379.47</v>
       </c>
     </row>
     <row r="24">
@@ -1458,22 +1458,22 @@
         </is>
       </c>
       <c r="F24">
-        <v>-92.43000000000001</v>
+        <v>-60.1</v>
       </c>
       <c r="G24">
-        <v>48.88</v>
+        <v>110.13</v>
       </c>
       <c r="H24">
-        <v>159.78</v>
+        <v>243.12</v>
       </c>
       <c r="I24">
-        <v>313.33</v>
+        <v>435.23</v>
       </c>
       <c r="J24">
-        <v>488.69</v>
+        <v>666.62</v>
       </c>
       <c r="K24">
-        <v>538.6</v>
+        <v>766.45</v>
       </c>
     </row>
     <row r="25">
@@ -1503,26 +1503,26 @@
         </is>
       </c>
       <c r="F25">
-        <v>-62.8</v>
+        <v>-40.8</v>
       </c>
       <c r="G25">
-        <v>29.9</v>
+        <v>67.3</v>
       </c>
       <c r="H25">
-        <v>72.09999999999999</v>
+        <v>109.7</v>
       </c>
       <c r="I25">
-        <v>102.2</v>
+        <v>141.9</v>
       </c>
       <c r="J25">
-        <v>119.2</v>
+        <v>162.6</v>
       </c>
       <c r="K25">
-        <v>87.90000000000001</v>
+        <v>125</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>GCAM 1.9x higher at 2050</t>
+          <t>GCAM 2.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -1598,22 +1598,22 @@
         </is>
       </c>
       <c r="F27">
-        <v>17.48</v>
+        <v>16.48</v>
       </c>
       <c r="G27">
-        <v>47.19</v>
+        <v>35.79</v>
       </c>
       <c r="H27">
-        <v>97.25</v>
+        <v>73.7</v>
       </c>
       <c r="I27">
-        <v>194.84</v>
+        <v>156.12</v>
       </c>
       <c r="J27">
-        <v>312.08</v>
+        <v>259.17</v>
       </c>
       <c r="K27">
-        <v>410.37</v>
+        <v>343.3</v>
       </c>
     </row>
     <row r="28">
@@ -1643,22 +1643,22 @@
         </is>
       </c>
       <c r="F28">
-        <v>2.42</v>
+        <v>1.42</v>
       </c>
       <c r="G28">
-        <v>33.59</v>
+        <v>22.19</v>
       </c>
       <c r="H28">
-        <v>63.66</v>
+        <v>40.11</v>
       </c>
       <c r="I28">
-        <v>156.49</v>
+        <v>117.76</v>
       </c>
       <c r="J28">
-        <v>191.21</v>
+        <v>138.3</v>
       </c>
       <c r="K28">
-        <v>249.14</v>
+        <v>182.06</v>
       </c>
     </row>
     <row r="29">
@@ -1688,26 +1688,26 @@
         </is>
       </c>
       <c r="F29">
-        <v>16.1</v>
+        <v>9.4</v>
       </c>
       <c r="G29">
-        <v>246.9</v>
+        <v>163.1</v>
       </c>
       <c r="H29">
-        <v>189.5</v>
+        <v>119.4</v>
       </c>
       <c r="I29">
-        <v>408</v>
+        <v>307</v>
       </c>
       <c r="J29">
-        <v>158.2</v>
+        <v>114.4</v>
       </c>
       <c r="K29">
-        <v>154.5</v>
+        <v>112.9</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>GCAM 2.5x higher at 2050</t>
+          <t>GCAM 2.1x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -1783,22 +1783,22 @@
         </is>
       </c>
       <c r="F31">
-        <v>1.81</v>
+        <v>1.55</v>
       </c>
       <c r="G31">
-        <v>4.28</v>
+        <v>3.23</v>
       </c>
       <c r="H31">
-        <v>7.89</v>
+        <v>6</v>
       </c>
       <c r="I31">
-        <v>15.51</v>
+        <v>12.1</v>
       </c>
       <c r="J31">
-        <v>26.6</v>
+        <v>21.3</v>
       </c>
       <c r="K31">
-        <v>38.29</v>
+        <v>30.92</v>
       </c>
     </row>
     <row r="32">
@@ -1828,22 +1828,22 @@
         </is>
       </c>
       <c r="F32">
-        <v>-1.43</v>
+        <v>-1.69</v>
       </c>
       <c r="G32">
-        <v>0.87</v>
+        <v>-0.18</v>
       </c>
       <c r="H32">
-        <v>4.29</v>
+        <v>2.39</v>
       </c>
       <c r="I32">
-        <v>11.64</v>
+        <v>8.23</v>
       </c>
       <c r="J32">
-        <v>26.38</v>
+        <v>21.08</v>
       </c>
       <c r="K32">
-        <v>34.7</v>
+        <v>27.33</v>
       </c>
     </row>
     <row r="33">
@@ -1873,26 +1873,26 @@
         </is>
       </c>
       <c r="F33">
-        <v>-44.2</v>
+        <v>-52.1</v>
       </c>
       <c r="G33">
-        <v>25.4</v>
+        <v>-5.3</v>
       </c>
       <c r="H33">
-        <v>118.9</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="I33">
-        <v>300.7</v>
+        <v>212.7</v>
       </c>
       <c r="J33">
-        <v>12152.3</v>
+        <v>9713.1</v>
       </c>
       <c r="K33">
-        <v>965.5</v>
+        <v>760.3</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>GCAM 10.7x higher at 2050</t>
+          <t>GCAM 8.6x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -1968,22 +1968,22 @@
         </is>
       </c>
       <c r="F35">
-        <v>223.68</v>
+        <v>220.22</v>
       </c>
       <c r="G35">
-        <v>266.13</v>
+        <v>253.44</v>
       </c>
       <c r="H35">
-        <v>314.46</v>
+        <v>294.93</v>
       </c>
       <c r="I35">
-        <v>378.79</v>
+        <v>352.8</v>
       </c>
       <c r="J35">
-        <v>460.9</v>
+        <v>428.48</v>
       </c>
       <c r="K35">
-        <v>546.3200000000001</v>
+        <v>508.14</v>
       </c>
     </row>
     <row r="36">
@@ -2013,22 +2013,22 @@
         </is>
       </c>
       <c r="F36">
-        <v>35.16</v>
+        <v>31.71</v>
       </c>
       <c r="G36">
-        <v>-39.33</v>
+        <v>-52.02</v>
       </c>
       <c r="H36">
-        <v>-58.95</v>
+        <v>-78.47</v>
       </c>
       <c r="I36">
-        <v>-95.72</v>
+        <v>-121.71</v>
       </c>
       <c r="J36">
-        <v>-116</v>
+        <v>-148.42</v>
       </c>
       <c r="K36">
-        <v>-187.96</v>
+        <v>-226.13</v>
       </c>
     </row>
     <row r="37">
@@ -2058,26 +2058,26 @@
         </is>
       </c>
       <c r="F37">
-        <v>18.7</v>
+        <v>16.8</v>
       </c>
       <c r="G37">
-        <v>-12.9</v>
+        <v>-17</v>
       </c>
       <c r="H37">
-        <v>-15.8</v>
+        <v>-21</v>
       </c>
       <c r="I37">
-        <v>-20.2</v>
+        <v>-25.7</v>
       </c>
       <c r="J37">
-        <v>-20.1</v>
+        <v>-25.7</v>
       </c>
       <c r="K37">
-        <v>-25.6</v>
+        <v>-30.8</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>MSG 1.3x higher at 2050</t>
+          <t>MSG 1.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -2153,22 +2153,22 @@
         </is>
       </c>
       <c r="F39">
-        <v>241.26</v>
+        <v>237.85</v>
       </c>
       <c r="G39">
-        <v>288.99</v>
+        <v>276.2</v>
       </c>
       <c r="H39">
-        <v>343.39</v>
+        <v>323.67</v>
       </c>
       <c r="I39">
-        <v>414.43</v>
+        <v>388.18</v>
       </c>
       <c r="J39">
-        <v>503.55</v>
+        <v>470.82</v>
       </c>
       <c r="K39">
-        <v>596.14</v>
+        <v>557.61</v>
       </c>
     </row>
     <row r="40">
@@ -2198,22 +2198,22 @@
         </is>
       </c>
       <c r="F40">
-        <v>38.21</v>
+        <v>34.79</v>
       </c>
       <c r="G40">
-        <v>-32.91</v>
+        <v>-45.7</v>
       </c>
       <c r="H40">
-        <v>-51.21</v>
+        <v>-70.92</v>
       </c>
       <c r="I40">
-        <v>-88.23999999999999</v>
+        <v>-114.49</v>
       </c>
       <c r="J40">
-        <v>-106.52</v>
+        <v>-139.25</v>
       </c>
       <c r="K40">
-        <v>-176.73</v>
+        <v>-215.26</v>
       </c>
     </row>
     <row r="41">
@@ -2243,26 +2243,26 @@
         </is>
       </c>
       <c r="F41">
-        <v>18.8</v>
+        <v>17.1</v>
       </c>
       <c r="G41">
-        <v>-10.2</v>
+        <v>-14.2</v>
       </c>
       <c r="H41">
-        <v>-13</v>
+        <v>-18</v>
       </c>
       <c r="I41">
-        <v>-17.6</v>
+        <v>-22.8</v>
       </c>
       <c r="J41">
-        <v>-17.5</v>
+        <v>-22.8</v>
       </c>
       <c r="K41">
-        <v>-22.9</v>
+        <v>-27.9</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>MSG 1.3x higher at 2050</t>
+          <t>MSG 1.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -2338,22 +2338,22 @@
         </is>
       </c>
       <c r="F43">
-        <v>59.21</v>
+        <v>57.14</v>
       </c>
       <c r="G43">
-        <v>74.94</v>
+        <v>66.67</v>
       </c>
       <c r="H43">
-        <v>92.5</v>
+        <v>78.39</v>
       </c>
       <c r="I43">
-        <v>123.19</v>
+        <v>101.38</v>
       </c>
       <c r="J43">
-        <v>161.84</v>
+        <v>131.81</v>
       </c>
       <c r="K43">
-        <v>196.07</v>
+        <v>158.28</v>
       </c>
     </row>
     <row r="44">
@@ -2383,22 +2383,22 @@
         </is>
       </c>
       <c r="F44">
-        <v>23.05</v>
+        <v>20.98</v>
       </c>
       <c r="G44">
-        <v>-49.88</v>
+        <v>-58.15</v>
       </c>
       <c r="H44">
-        <v>-84.95999999999999</v>
+        <v>-99.06999999999999</v>
       </c>
       <c r="I44">
-        <v>-117.08</v>
+        <v>-138.89</v>
       </c>
       <c r="J44">
-        <v>-143.32</v>
+        <v>-173.35</v>
       </c>
       <c r="K44">
-        <v>-184.67</v>
+        <v>-222.46</v>
       </c>
     </row>
     <row r="45">
@@ -2428,26 +2428,26 @@
         </is>
       </c>
       <c r="F45">
-        <v>63.7</v>
+        <v>58</v>
       </c>
       <c r="G45">
-        <v>-40</v>
+        <v>-46.6</v>
       </c>
       <c r="H45">
-        <v>-47.9</v>
+        <v>-55.8</v>
       </c>
       <c r="I45">
-        <v>-48.7</v>
+        <v>-57.8</v>
       </c>
       <c r="J45">
-        <v>-47</v>
+        <v>-56.8</v>
       </c>
       <c r="K45">
-        <v>-48.5</v>
+        <v>-58.4</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>MSG 1.9x higher at 2050</t>
+          <t>MSG 2.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -2523,22 +2523,22 @@
         </is>
       </c>
       <c r="F47">
-        <v>100.14</v>
+        <v>100.02</v>
       </c>
       <c r="G47">
-        <v>123.08</v>
+        <v>123.49</v>
       </c>
       <c r="H47">
-        <v>151.31</v>
+        <v>152.59</v>
       </c>
       <c r="I47">
-        <v>184.05</v>
+        <v>186.67</v>
       </c>
       <c r="J47">
-        <v>220.99</v>
+        <v>225.43</v>
       </c>
       <c r="K47">
-        <v>263.79</v>
+        <v>270</v>
       </c>
     </row>
     <row r="48">
@@ -2568,22 +2568,22 @@
         </is>
       </c>
       <c r="F48">
-        <v>55.41</v>
+        <v>55.29</v>
       </c>
       <c r="G48">
-        <v>68.11</v>
+        <v>68.53</v>
       </c>
       <c r="H48">
-        <v>82.67</v>
+        <v>83.95</v>
       </c>
       <c r="I48">
-        <v>92.8</v>
+        <v>95.43000000000001</v>
       </c>
       <c r="J48">
-        <v>105.05</v>
+        <v>109.48</v>
       </c>
       <c r="K48">
-        <v>109.04</v>
+        <v>115.25</v>
       </c>
     </row>
     <row r="49">
@@ -2613,22 +2613,22 @@
         </is>
       </c>
       <c r="F49">
-        <v>123.9</v>
+        <v>123.6</v>
       </c>
       <c r="G49">
-        <v>123.9</v>
+        <v>124.7</v>
       </c>
       <c r="H49">
-        <v>120.4</v>
+        <v>122.3</v>
       </c>
       <c r="I49">
-        <v>101.7</v>
+        <v>104.6</v>
       </c>
       <c r="J49">
-        <v>90.59999999999999</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="K49">
-        <v>70.5</v>
+        <v>74.5</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -2708,22 +2708,22 @@
         </is>
       </c>
       <c r="F51">
-        <v>54.15</v>
+        <v>53.21</v>
       </c>
       <c r="G51">
-        <v>56.29</v>
+        <v>50.88</v>
       </c>
       <c r="H51">
-        <v>56.91</v>
+        <v>49.11</v>
       </c>
       <c r="I51">
-        <v>55.15</v>
+        <v>46.75</v>
       </c>
       <c r="J51">
-        <v>57.6</v>
+        <v>48.66</v>
       </c>
       <c r="K51">
-        <v>61.54</v>
+        <v>52.31</v>
       </c>
     </row>
     <row r="52">
@@ -2753,22 +2753,22 @@
         </is>
       </c>
       <c r="F52">
-        <v>-1.28</v>
+        <v>-2.22</v>
       </c>
       <c r="G52">
-        <v>-15.79</v>
+        <v>-21.2</v>
       </c>
       <c r="H52">
-        <v>1.68</v>
+        <v>-6.11</v>
       </c>
       <c r="I52">
-        <v>0.68</v>
+        <v>-7.72</v>
       </c>
       <c r="J52">
-        <v>14.79</v>
+        <v>5.85</v>
       </c>
       <c r="K52">
-        <v>0.08</v>
+        <v>-9.15</v>
       </c>
     </row>
     <row r="53">
@@ -2798,26 +2798,26 @@
         </is>
       </c>
       <c r="F53">
-        <v>-2.3</v>
+        <v>-4</v>
       </c>
       <c r="G53">
-        <v>-21.9</v>
+        <v>-29.4</v>
       </c>
       <c r="H53">
-        <v>3</v>
+        <v>-11.1</v>
       </c>
       <c r="I53">
-        <v>1.3</v>
+        <v>-14.2</v>
       </c>
       <c r="J53">
-        <v>34.5</v>
+        <v>13.7</v>
       </c>
       <c r="K53">
-        <v>0.1</v>
+        <v>-14.9</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>~0% gap at 2050</t>
+          <t>MSG 1.2x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -2893,22 +2893,22 @@
         </is>
       </c>
       <c r="F55">
-        <v>23.22</v>
+        <v>22.91</v>
       </c>
       <c r="G55">
-        <v>27.89</v>
+        <v>28.88</v>
       </c>
       <c r="H55">
-        <v>33.54</v>
+        <v>35.38</v>
       </c>
       <c r="I55">
-        <v>40.54</v>
+        <v>43.07</v>
       </c>
       <c r="J55">
-        <v>49.34</v>
+        <v>52.54</v>
       </c>
       <c r="K55">
-        <v>58.82</v>
+        <v>62.58</v>
       </c>
     </row>
     <row r="56">
@@ -2938,22 +2938,22 @@
         </is>
       </c>
       <c r="F56">
-        <v>2.14</v>
+        <v>1.83</v>
       </c>
       <c r="G56">
-        <v>-1.75</v>
+        <v>-0.76</v>
       </c>
       <c r="H56">
-        <v>-10.07</v>
+        <v>-8.23</v>
       </c>
       <c r="I56">
-        <v>-10.95</v>
+        <v>-8.42</v>
       </c>
       <c r="J56">
-        <v>-18.66</v>
+        <v>-15.46</v>
       </c>
       <c r="K56">
-        <v>-24.28</v>
+        <v>-20.52</v>
       </c>
     </row>
     <row r="57">
@@ -2983,26 +2983,26 @@
         </is>
       </c>
       <c r="F57">
-        <v>10.2</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G57">
-        <v>-5.9</v>
+        <v>-2.6</v>
       </c>
       <c r="H57">
-        <v>-23.1</v>
+        <v>-18.9</v>
       </c>
       <c r="I57">
-        <v>-21.3</v>
+        <v>-16.4</v>
       </c>
       <c r="J57">
-        <v>-27.4</v>
+        <v>-22.7</v>
       </c>
       <c r="K57">
-        <v>-29.2</v>
+        <v>-24.7</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>MSG 1.4x higher at 2050</t>
+          <t>MSG 1.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -3078,22 +3078,22 @@
         </is>
       </c>
       <c r="F59">
-        <v>574.09</v>
+        <v>570.54</v>
       </c>
       <c r="G59">
-        <v>663.38</v>
+        <v>649.51</v>
       </c>
       <c r="H59">
-        <v>764.78</v>
+        <v>743.4400000000001</v>
       </c>
       <c r="I59">
-        <v>888.91</v>
+        <v>860.58</v>
       </c>
       <c r="J59">
-        <v>1037.69</v>
+        <v>1002.68</v>
       </c>
       <c r="K59">
-        <v>1198.62</v>
+        <v>1157.79</v>
       </c>
     </row>
     <row r="60">
@@ -3123,22 +3123,22 @@
         </is>
       </c>
       <c r="F60">
-        <v>327.85</v>
+        <v>324.3</v>
       </c>
       <c r="G60">
-        <v>292.6</v>
+        <v>278.73</v>
       </c>
       <c r="H60">
-        <v>314.75</v>
+        <v>293.4</v>
       </c>
       <c r="I60">
-        <v>321.98</v>
+        <v>293.64</v>
       </c>
       <c r="J60">
-        <v>353.2</v>
+        <v>318.19</v>
       </c>
       <c r="K60">
-        <v>338.8</v>
+        <v>297.97</v>
       </c>
     </row>
     <row r="61">
@@ -3168,26 +3168,26 @@
         </is>
       </c>
       <c r="F61">
-        <v>133.1</v>
+        <v>131.7</v>
       </c>
       <c r="G61">
-        <v>78.90000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="H61">
-        <v>69.90000000000001</v>
+        <v>65.2</v>
       </c>
       <c r="I61">
-        <v>56.8</v>
+        <v>51.8</v>
       </c>
       <c r="J61">
-        <v>51.6</v>
+        <v>46.5</v>
       </c>
       <c r="K61">
-        <v>39.4</v>
+        <v>34.7</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>GCAM 1.4x higher at 2050</t>
+          <t>GCAM 1.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -3245,22 +3245,22 @@
         </is>
       </c>
       <c r="F63">
-        <v>303</v>
+        <v>299.43</v>
       </c>
       <c r="G63">
-        <v>362.27</v>
+        <v>348.48</v>
       </c>
       <c r="H63">
-        <v>427</v>
+        <v>405.77</v>
       </c>
       <c r="I63">
-        <v>511.34</v>
+        <v>483.2</v>
       </c>
       <c r="J63">
-        <v>618.54</v>
+        <v>583.67</v>
       </c>
       <c r="K63">
-        <v>733.84</v>
+        <v>692.98</v>
       </c>
     </row>
     <row r="64">
@@ -3394,22 +3394,22 @@
         </is>
       </c>
       <c r="F67">
-        <v>4399.98</v>
+        <v>4390.92</v>
       </c>
       <c r="G67">
-        <v>4868.43</v>
+        <v>4807.47</v>
       </c>
       <c r="H67">
-        <v>5481.38</v>
+        <v>5395.87</v>
       </c>
       <c r="I67">
-        <v>6246.89</v>
+        <v>6156.05</v>
       </c>
       <c r="J67">
-        <v>7252.72</v>
+        <v>7159.58</v>
       </c>
       <c r="K67">
-        <v>8466.790000000001</v>
+        <v>8371.51</v>
       </c>
     </row>
     <row r="68">
@@ -3439,22 +3439,22 @@
         </is>
       </c>
       <c r="F68">
-        <v>1357.4</v>
+        <v>1348.34</v>
       </c>
       <c r="G68">
-        <v>884.98</v>
+        <v>824.03</v>
       </c>
       <c r="H68">
-        <v>827.9400000000001</v>
+        <v>742.4299999999999</v>
       </c>
       <c r="I68">
-        <v>619.9</v>
+        <v>529.0599999999999</v>
       </c>
       <c r="J68">
-        <v>549.36</v>
+        <v>456.22</v>
       </c>
       <c r="K68">
-        <v>85.06</v>
+        <v>-10.21</v>
       </c>
     </row>
     <row r="69">
@@ -3484,26 +3484,26 @@
         </is>
       </c>
       <c r="F69">
-        <v>44.6</v>
+        <v>44.3</v>
       </c>
       <c r="G69">
-        <v>22.2</v>
+        <v>20.7</v>
       </c>
       <c r="H69">
-        <v>17.8</v>
+        <v>16</v>
       </c>
       <c r="I69">
-        <v>11</v>
+        <v>9.4</v>
       </c>
       <c r="J69">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
       <c r="K69">
-        <v>1</v>
+        <v>-0.1</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>~1% gap at 2050</t>
+          <t>~0% gap at 2050</t>
         </is>
       </c>
     </row>
@@ -3579,22 +3579,22 @@
         </is>
       </c>
       <c r="F71">
-        <v>1340.62</v>
+        <v>1340.6</v>
       </c>
       <c r="G71">
-        <v>1670.84</v>
+        <v>1671.64</v>
       </c>
       <c r="H71">
-        <v>2081.82</v>
+        <v>2084.14</v>
       </c>
       <c r="I71">
-        <v>2572.74</v>
+        <v>2577.34</v>
       </c>
       <c r="J71">
-        <v>3140.9</v>
+        <v>3149.3</v>
       </c>
       <c r="K71">
-        <v>3794.14</v>
+        <v>3805.85</v>
       </c>
     </row>
     <row r="72">
@@ -3624,22 +3624,22 @@
         </is>
       </c>
       <c r="F72">
-        <v>150.7</v>
+        <v>150.69</v>
       </c>
       <c r="G72">
-        <v>163.88</v>
+        <v>164.69</v>
       </c>
       <c r="H72">
-        <v>115.82</v>
+        <v>118.15</v>
       </c>
       <c r="I72">
-        <v>-58.24</v>
+        <v>-53.63</v>
       </c>
       <c r="J72">
-        <v>-40.54</v>
+        <v>-32.14</v>
       </c>
       <c r="K72">
-        <v>-30.75</v>
+        <v>-19.04</v>
       </c>
     </row>
     <row r="73">
@@ -3675,20 +3675,20 @@
         <v>10.9</v>
       </c>
       <c r="H73">
-        <v>5.9</v>
+        <v>6</v>
       </c>
       <c r="I73">
-        <v>-2.2</v>
+        <v>-2</v>
       </c>
       <c r="J73">
-        <v>-1.3</v>
+        <v>-1</v>
       </c>
       <c r="K73">
-        <v>-0.8</v>
+        <v>-0.5</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>~1% gap at 2050</t>
+          <t>~0% gap at 2050</t>
         </is>
       </c>
     </row>
@@ -3764,22 +3764,22 @@
         </is>
       </c>
       <c r="F75">
-        <v>2129.78</v>
+        <v>2129.48</v>
       </c>
       <c r="G75">
-        <v>2197.96</v>
+        <v>2199.72</v>
       </c>
       <c r="H75">
-        <v>2330.86</v>
+        <v>2333.27</v>
       </c>
       <c r="I75">
-        <v>2544.65</v>
+        <v>2546.61</v>
       </c>
       <c r="J75">
-        <v>2856.93</v>
+        <v>2858.71</v>
       </c>
       <c r="K75">
-        <v>3257.38</v>
+        <v>3257.7</v>
       </c>
     </row>
     <row r="76">
@@ -3809,22 +3809,22 @@
         </is>
       </c>
       <c r="F76">
-        <v>1053.64</v>
+        <v>1053.34</v>
       </c>
       <c r="G76">
-        <v>725.7</v>
+        <v>727.45</v>
       </c>
       <c r="H76">
-        <v>544.6</v>
+        <v>547</v>
       </c>
       <c r="I76">
-        <v>510.7</v>
+        <v>512.66</v>
       </c>
       <c r="J76">
-        <v>310.58</v>
+        <v>312.35</v>
       </c>
       <c r="K76">
-        <v>189.79</v>
+        <v>190.12</v>
       </c>
     </row>
     <row r="77">
@@ -3857,16 +3857,16 @@
         <v>97.90000000000001</v>
       </c>
       <c r="G77">
-        <v>49.3</v>
+        <v>49.4</v>
       </c>
       <c r="H77">
-        <v>30.5</v>
+        <v>30.6</v>
       </c>
       <c r="I77">
-        <v>25.1</v>
+        <v>25.2</v>
       </c>
       <c r="J77">
-        <v>12.2</v>
+        <v>12.3</v>
       </c>
       <c r="K77">
         <v>6.2</v>
@@ -3949,22 +3949,22 @@
         </is>
       </c>
       <c r="F79">
-        <v>780.5599999999999</v>
+        <v>771.8200000000001</v>
       </c>
       <c r="G79">
-        <v>829.4299999999999</v>
+        <v>765.89</v>
       </c>
       <c r="H79">
-        <v>874.21</v>
+        <v>783.92</v>
       </c>
       <c r="I79">
-        <v>902.97</v>
+        <v>805.49</v>
       </c>
       <c r="J79">
-        <v>988.72</v>
+        <v>885.3200000000001</v>
       </c>
       <c r="K79">
-        <v>1102.1</v>
+        <v>994.67</v>
       </c>
     </row>
     <row r="80">
@@ -3994,22 +3994,22 @@
         </is>
       </c>
       <c r="F80">
-        <v>4.02</v>
+        <v>-4.71</v>
       </c>
       <c r="G80">
-        <v>-174.8</v>
+        <v>-238.34</v>
       </c>
       <c r="H80">
-        <v>-26.97</v>
+        <v>-117.26</v>
       </c>
       <c r="I80">
-        <v>-59.1</v>
+        <v>-156.58</v>
       </c>
       <c r="J80">
-        <v>13.17</v>
+        <v>-90.23999999999999</v>
       </c>
       <c r="K80">
-        <v>-387.15</v>
+        <v>-494.58</v>
       </c>
     </row>
     <row r="81">
@@ -4039,26 +4039,26 @@
         </is>
       </c>
       <c r="F81">
-        <v>0.5</v>
+        <v>-0.6</v>
       </c>
       <c r="G81">
-        <v>-17.4</v>
+        <v>-23.7</v>
       </c>
       <c r="H81">
-        <v>-3</v>
+        <v>-13</v>
       </c>
       <c r="I81">
-        <v>-6.1</v>
+        <v>-16.3</v>
       </c>
       <c r="J81">
-        <v>1.3</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="K81">
-        <v>-26</v>
+        <v>-33.2</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>MSG 1.4x higher at 2050</t>
+          <t>MSG 1.5x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -4134,22 +4134,22 @@
         </is>
       </c>
       <c r="F83">
-        <v>586.08</v>
+        <v>597.86</v>
       </c>
       <c r="G83">
-        <v>776.79</v>
+        <v>764.58</v>
       </c>
       <c r="H83">
-        <v>1026.37</v>
+        <v>993.61</v>
       </c>
       <c r="I83">
-        <v>1364.72</v>
+        <v>1303.72</v>
       </c>
       <c r="J83">
-        <v>1786.34</v>
+        <v>1693.02</v>
       </c>
       <c r="K83">
-        <v>2291.05</v>
+        <v>2165.97</v>
       </c>
     </row>
     <row r="84">
@@ -4179,22 +4179,22 @@
         </is>
       </c>
       <c r="F84">
-        <v>111.46</v>
+        <v>123.25</v>
       </c>
       <c r="G84">
-        <v>-65.81</v>
+        <v>-78.02</v>
       </c>
       <c r="H84">
-        <v>-215.61</v>
+        <v>-248.36</v>
       </c>
       <c r="I84">
-        <v>-293.15</v>
+        <v>-354.14</v>
       </c>
       <c r="J84">
-        <v>-421.82</v>
+        <v>-515.14</v>
       </c>
       <c r="K84">
-        <v>-613.0599999999999</v>
+        <v>-738.14</v>
       </c>
     </row>
     <row r="85">
@@ -4224,22 +4224,22 @@
         </is>
       </c>
       <c r="F85">
-        <v>23.5</v>
+        <v>26</v>
       </c>
       <c r="G85">
-        <v>-7.8</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="H85">
-        <v>-17.4</v>
+        <v>-20</v>
       </c>
       <c r="I85">
-        <v>-17.7</v>
+        <v>-21.4</v>
       </c>
       <c r="J85">
-        <v>-19.1</v>
+        <v>-23.3</v>
       </c>
       <c r="K85">
-        <v>-21.1</v>
+        <v>-25.4</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
@@ -4319,22 +4319,22 @@
         </is>
       </c>
       <c r="F87">
-        <v>917.27</v>
+        <v>908.35</v>
       </c>
       <c r="G87">
-        <v>1060.24</v>
+        <v>1074.59</v>
       </c>
       <c r="H87">
-        <v>1211.88</v>
+        <v>1240.91</v>
       </c>
       <c r="I87">
-        <v>1365.17</v>
+        <v>1410.11</v>
       </c>
       <c r="J87">
-        <v>1550.47</v>
+        <v>1613.59</v>
       </c>
       <c r="K87">
-        <v>1765.67</v>
+        <v>1842.62</v>
       </c>
     </row>
     <row r="88">
@@ -4364,22 +4364,22 @@
         </is>
       </c>
       <c r="F88">
-        <v>-45.49</v>
+        <v>-54.42</v>
       </c>
       <c r="G88">
-        <v>45.96</v>
+        <v>60.3</v>
       </c>
       <c r="H88">
-        <v>35.28</v>
+        <v>64.31</v>
       </c>
       <c r="I88">
-        <v>55.05</v>
+        <v>99.98999999999999</v>
       </c>
       <c r="J88">
-        <v>186.36</v>
+        <v>249.48</v>
       </c>
       <c r="K88">
-        <v>432.91</v>
+        <v>509.86</v>
       </c>
     </row>
     <row r="89">
@@ -4409,26 +4409,26 @@
         </is>
       </c>
       <c r="F89">
-        <v>-4.7</v>
+        <v>-5.7</v>
       </c>
       <c r="G89">
-        <v>4.5</v>
+        <v>5.9</v>
       </c>
       <c r="H89">
-        <v>3</v>
+        <v>5.5</v>
       </c>
       <c r="I89">
-        <v>4.2</v>
+        <v>7.6</v>
       </c>
       <c r="J89">
-        <v>13.7</v>
+        <v>18.3</v>
       </c>
       <c r="K89">
-        <v>32.5</v>
+        <v>38.3</v>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>GCAM 1.3x higher at 2050</t>
+          <t>GCAM 1.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -4504,22 +4504,22 @@
         </is>
       </c>
       <c r="F91">
-        <v>879.0700000000001</v>
+        <v>868.41</v>
       </c>
       <c r="G91">
-        <v>966.78</v>
+        <v>900.04</v>
       </c>
       <c r="H91">
-        <v>1058.61</v>
+        <v>966.9400000000001</v>
       </c>
       <c r="I91">
-        <v>1146.55</v>
+        <v>1052.62</v>
       </c>
       <c r="J91">
-        <v>1310.4</v>
+        <v>1215.02</v>
       </c>
       <c r="K91">
-        <v>1515.11</v>
+        <v>1421.39</v>
       </c>
     </row>
     <row r="92">
@@ -4549,22 +4549,22 @@
         </is>
       </c>
       <c r="F92">
-        <v>56.74</v>
+        <v>46.09</v>
       </c>
       <c r="G92">
-        <v>-172.54</v>
+        <v>-239.29</v>
       </c>
       <c r="H92">
-        <v>-0.71</v>
+        <v>-92.38</v>
       </c>
       <c r="I92">
-        <v>-84.98999999999999</v>
+        <v>-178.92</v>
       </c>
       <c r="J92">
-        <v>-54.68</v>
+        <v>-150.06</v>
       </c>
       <c r="K92">
-        <v>-527.03</v>
+        <v>-620.74</v>
       </c>
     </row>
     <row r="93">
@@ -4594,26 +4594,26 @@
         </is>
       </c>
       <c r="F93">
-        <v>6.9</v>
+        <v>5.6</v>
       </c>
       <c r="G93">
-        <v>-15.1</v>
+        <v>-21</v>
       </c>
       <c r="H93">
-        <v>-0.1</v>
+        <v>-8.699999999999999</v>
       </c>
       <c r="I93">
-        <v>-6.9</v>
+        <v>-14.5</v>
       </c>
       <c r="J93">
-        <v>-4</v>
+        <v>-11</v>
       </c>
       <c r="K93">
-        <v>-25.8</v>
+        <v>-30.4</v>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>MSG 1.3x higher at 2050</t>
+          <t>MSG 1.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -4689,22 +4689,22 @@
         </is>
       </c>
       <c r="F95">
-        <v>477.64</v>
+        <v>477.1</v>
       </c>
       <c r="G95">
-        <v>606.33</v>
+        <v>608.09</v>
       </c>
       <c r="H95">
-        <v>770.16</v>
+        <v>775.97</v>
       </c>
       <c r="I95">
-        <v>970.27</v>
+        <v>982.92</v>
       </c>
       <c r="J95">
-        <v>1199.61</v>
+        <v>1221.51</v>
       </c>
       <c r="K95">
-        <v>1461.23</v>
+        <v>1492.86</v>
       </c>
     </row>
     <row r="96">
@@ -4734,22 +4734,22 @@
         </is>
       </c>
       <c r="F96">
-        <v>246.69</v>
+        <v>246.15</v>
       </c>
       <c r="G96">
-        <v>273.28</v>
+        <v>275.04</v>
       </c>
       <c r="H96">
-        <v>312.28</v>
+        <v>318.09</v>
       </c>
       <c r="I96">
-        <v>342.02</v>
+        <v>354.67</v>
       </c>
       <c r="J96">
-        <v>332.9</v>
+        <v>354.8</v>
       </c>
       <c r="K96">
-        <v>267.54</v>
+        <v>299.17</v>
       </c>
     </row>
     <row r="97">
@@ -4779,26 +4779,26 @@
         </is>
       </c>
       <c r="F97">
-        <v>106.8</v>
+        <v>106.6</v>
       </c>
       <c r="G97">
-        <v>82.09999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="H97">
-        <v>68.2</v>
+        <v>69.5</v>
       </c>
       <c r="I97">
-        <v>54.4</v>
+        <v>56.5</v>
       </c>
       <c r="J97">
-        <v>38.4</v>
+        <v>40.9</v>
       </c>
       <c r="K97">
-        <v>22.4</v>
+        <v>25.1</v>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>GCAM 1.2x higher at 2050</t>
+          <t>GCAM 1.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -4874,22 +4874,22 @@
         </is>
       </c>
       <c r="F99">
-        <v>1539.79</v>
+        <v>1539.07</v>
       </c>
       <c r="G99">
-        <v>1454.66</v>
+        <v>1456.68</v>
       </c>
       <c r="H99">
-        <v>1401.91</v>
+        <v>1406.91</v>
       </c>
       <c r="I99">
-        <v>1368.2</v>
+        <v>1377.27</v>
       </c>
       <c r="J99">
-        <v>1350.66</v>
+        <v>1364.78</v>
       </c>
       <c r="K99">
-        <v>1352.72</v>
+        <v>1371.95</v>
       </c>
     </row>
     <row r="100">
@@ -4919,22 +4919,22 @@
         </is>
       </c>
       <c r="F100">
-        <v>1003.69</v>
+        <v>1002.96</v>
       </c>
       <c r="G100">
-        <v>846.53</v>
+        <v>848.55</v>
       </c>
       <c r="H100">
-        <v>787.5</v>
+        <v>792.49</v>
       </c>
       <c r="I100">
-        <v>754.67</v>
+        <v>763.74</v>
       </c>
       <c r="J100">
-        <v>719.29</v>
+        <v>733.41</v>
       </c>
       <c r="K100">
-        <v>711.62</v>
+        <v>730.85</v>
       </c>
     </row>
     <row r="101">
@@ -4964,22 +4964,22 @@
         </is>
       </c>
       <c r="F101">
-        <v>187.2</v>
+        <v>187.1</v>
       </c>
       <c r="G101">
-        <v>139.2</v>
+        <v>139.5</v>
       </c>
       <c r="H101">
-        <v>128.2</v>
+        <v>129</v>
       </c>
       <c r="I101">
-        <v>123</v>
+        <v>124.5</v>
       </c>
       <c r="J101">
-        <v>113.9</v>
+        <v>116.2</v>
       </c>
       <c r="K101">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="L101" t="inlineStr">
         <is>
@@ -5059,22 +5059,22 @@
         </is>
       </c>
       <c r="F103">
-        <v>52.1</v>
+        <v>57.36</v>
       </c>
       <c r="G103">
-        <v>71.73999999999999</v>
+        <v>80.56</v>
       </c>
       <c r="H103">
-        <v>106.48</v>
+        <v>119.03</v>
       </c>
       <c r="I103">
-        <v>151.2</v>
+        <v>163.46</v>
       </c>
       <c r="J103">
-        <v>195.37</v>
+        <v>207.21</v>
       </c>
       <c r="K103">
-        <v>246.12</v>
+        <v>256.53</v>
       </c>
     </row>
     <row r="104">
@@ -5104,22 +5104,22 @@
         </is>
       </c>
       <c r="F104">
-        <v>51.82</v>
+        <v>57.09</v>
       </c>
       <c r="G104">
-        <v>61.23</v>
+        <v>70.05</v>
       </c>
       <c r="H104">
-        <v>-39.83</v>
+        <v>-27.29</v>
       </c>
       <c r="I104">
-        <v>-68.45</v>
+        <v>-56.18</v>
       </c>
       <c r="J104">
-        <v>-196.67</v>
+        <v>-184.83</v>
       </c>
       <c r="K104">
-        <v>-405.43</v>
+        <v>-395.01</v>
       </c>
     </row>
     <row r="105">
@@ -5149,26 +5149,26 @@
         </is>
       </c>
       <c r="F105">
-        <v>18702.5</v>
+        <v>20603.4</v>
       </c>
       <c r="G105">
-        <v>582.4</v>
+        <v>666.4</v>
       </c>
       <c r="H105">
-        <v>-27.2</v>
+        <v>-18.7</v>
       </c>
       <c r="I105">
-        <v>-31.2</v>
+        <v>-25.6</v>
       </c>
       <c r="J105">
-        <v>-50.2</v>
+        <v>-47.1</v>
       </c>
       <c r="K105">
-        <v>-62.2</v>
+        <v>-60.6</v>
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>MSG 2.6x higher at 2050</t>
+          <t>MSG 2.5x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -5244,22 +5244,22 @@
         </is>
       </c>
       <c r="F107">
-        <v>688.13</v>
+        <v>678.4400000000001</v>
       </c>
       <c r="G107">
-        <v>720.26</v>
+        <v>651.92</v>
       </c>
       <c r="H107">
-        <v>730.66</v>
+        <v>635.3200000000001</v>
       </c>
       <c r="I107">
-        <v>709.09</v>
+        <v>609.51</v>
       </c>
       <c r="J107">
-        <v>740.1</v>
+        <v>637.22</v>
       </c>
       <c r="K107">
-        <v>787.01</v>
+        <v>683.54</v>
       </c>
     </row>
     <row r="108">
@@ -5289,22 +5289,22 @@
         </is>
       </c>
       <c r="F108">
-        <v>-0.2</v>
+        <v>-9.890000000000001</v>
       </c>
       <c r="G108">
-        <v>-225.57</v>
+        <v>-293.91</v>
       </c>
       <c r="H108">
-        <v>-15.16</v>
+        <v>-110.5</v>
       </c>
       <c r="I108">
-        <v>-33.33</v>
+        <v>-132.91</v>
       </c>
       <c r="J108">
-        <v>156.59</v>
+        <v>53.71</v>
       </c>
       <c r="K108">
-        <v>-50.7</v>
+        <v>-154.16</v>
       </c>
     </row>
     <row r="109">
@@ -5334,26 +5334,26 @@
         </is>
       </c>
       <c r="F109">
-        <v>-0</v>
+        <v>-1.4</v>
       </c>
       <c r="G109">
-        <v>-23.8</v>
+        <v>-31.1</v>
       </c>
       <c r="H109">
-        <v>-2</v>
+        <v>-14.8</v>
       </c>
       <c r="I109">
-        <v>-4.5</v>
+        <v>-17.9</v>
       </c>
       <c r="J109">
-        <v>26.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K109">
-        <v>-6.1</v>
+        <v>-18.4</v>
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>MSG 1.1x higher at 2050</t>
+          <t>MSG 1.2x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -5429,22 +5429,22 @@
         </is>
       </c>
       <c r="F111">
-        <v>750.11</v>
+        <v>742.12</v>
       </c>
       <c r="G111">
-        <v>929.65</v>
+        <v>894.15</v>
       </c>
       <c r="H111">
-        <v>1170</v>
+        <v>1113.83</v>
       </c>
       <c r="I111">
-        <v>1485.29</v>
+        <v>1404.37</v>
       </c>
       <c r="J111">
-        <v>1871.93</v>
+        <v>1760.29</v>
       </c>
       <c r="K111">
-        <v>2339.44</v>
+        <v>2186.12</v>
       </c>
     </row>
     <row r="112">
@@ -5474,22 +5474,22 @@
         </is>
       </c>
       <c r="F112">
-        <v>426.59</v>
+        <v>418.61</v>
       </c>
       <c r="G112">
-        <v>359.51</v>
+        <v>324.01</v>
       </c>
       <c r="H112">
-        <v>370.35</v>
+        <v>314.19</v>
       </c>
       <c r="I112">
-        <v>509.13</v>
+        <v>428.21</v>
       </c>
       <c r="J112">
-        <v>706.89</v>
+        <v>595.25</v>
       </c>
       <c r="K112">
-        <v>827.36</v>
+        <v>674.03</v>
       </c>
     </row>
     <row r="113">
@@ -5519,26 +5519,26 @@
         </is>
       </c>
       <c r="F113">
-        <v>131.9</v>
+        <v>129.4</v>
       </c>
       <c r="G113">
-        <v>63.1</v>
+        <v>56.8</v>
       </c>
       <c r="H113">
-        <v>46.3</v>
+        <v>39.3</v>
       </c>
       <c r="I113">
-        <v>52.2</v>
+        <v>43.9</v>
       </c>
       <c r="J113">
-        <v>60.7</v>
+        <v>51.1</v>
       </c>
       <c r="K113">
-        <v>54.7</v>
+        <v>44.6</v>
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>GCAM 1.5x higher at 2050</t>
+          <t>GCAM 1.4x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -5614,22 +5614,22 @@
         </is>
       </c>
       <c r="F115">
-        <v>1385.75</v>
+        <v>1363.38</v>
       </c>
       <c r="G115">
-        <v>1588.58</v>
+        <v>1560.5</v>
       </c>
       <c r="H115">
-        <v>1833.88</v>
+        <v>1798.93</v>
       </c>
       <c r="I115">
-        <v>2121.05</v>
+        <v>2075.07</v>
       </c>
       <c r="J115">
-        <v>2497.75</v>
+        <v>2436.57</v>
       </c>
       <c r="K115">
-        <v>2953.77</v>
+        <v>2868.38</v>
       </c>
     </row>
     <row r="116">
@@ -5659,22 +5659,22 @@
         </is>
       </c>
       <c r="F116">
-        <v>9.32</v>
+        <v>-13.05</v>
       </c>
       <c r="G116">
-        <v>68.25</v>
+        <v>40.18</v>
       </c>
       <c r="H116">
-        <v>-251.58</v>
+        <v>-286.52</v>
       </c>
       <c r="I116">
-        <v>-461.1</v>
+        <v>-507.07</v>
       </c>
       <c r="J116">
-        <v>-587.89</v>
+        <v>-649.0700000000001</v>
       </c>
       <c r="K116">
-        <v>-654.66</v>
+        <v>-740.05</v>
       </c>
     </row>
     <row r="117">
@@ -5704,26 +5704,26 @@
         </is>
       </c>
       <c r="F117">
-        <v>0.7</v>
+        <v>-0.9</v>
       </c>
       <c r="G117">
-        <v>4.5</v>
+        <v>2.6</v>
       </c>
       <c r="H117">
-        <v>-12.1</v>
+        <v>-13.7</v>
       </c>
       <c r="I117">
-        <v>-17.9</v>
+        <v>-19.6</v>
       </c>
       <c r="J117">
-        <v>-19.1</v>
+        <v>-21</v>
       </c>
       <c r="K117">
-        <v>-18.1</v>
+        <v>-20.5</v>
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>MSG 1.2x higher at 2050</t>
+          <t>MSG 1.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -5799,22 +5799,22 @@
         </is>
       </c>
       <c r="F119">
-        <v>1075.24</v>
+        <v>1054.06</v>
       </c>
       <c r="G119">
-        <v>1175.34</v>
+        <v>1087.54</v>
       </c>
       <c r="H119">
-        <v>1282.03</v>
+        <v>1158.21</v>
       </c>
       <c r="I119">
-        <v>1396.75</v>
+        <v>1254.71</v>
       </c>
       <c r="J119">
-        <v>1593.3</v>
+        <v>1434.84</v>
       </c>
       <c r="K119">
-        <v>1823.33</v>
+        <v>1656.32</v>
       </c>
     </row>
     <row r="120">
@@ -5844,22 +5844,22 @@
         </is>
       </c>
       <c r="F120">
-        <v>221.8</v>
+        <v>200.62</v>
       </c>
       <c r="G120">
-        <v>-592.49</v>
+        <v>-680.29</v>
       </c>
       <c r="H120">
-        <v>-264.56</v>
+        <v>-388.39</v>
       </c>
       <c r="I120">
-        <v>-388.27</v>
+        <v>-530.3099999999999</v>
       </c>
       <c r="J120">
-        <v>-343.13</v>
+        <v>-501.6</v>
       </c>
       <c r="K120">
-        <v>-693.8200000000001</v>
+        <v>-860.83</v>
       </c>
     </row>
     <row r="121">
@@ -5889,26 +5889,26 @@
         </is>
       </c>
       <c r="F121">
-        <v>26</v>
+        <v>23.5</v>
       </c>
       <c r="G121">
-        <v>-33.5</v>
+        <v>-38.5</v>
       </c>
       <c r="H121">
-        <v>-17.1</v>
+        <v>-25.1</v>
       </c>
       <c r="I121">
-        <v>-21.8</v>
+        <v>-29.7</v>
       </c>
       <c r="J121">
-        <v>-17.7</v>
+        <v>-25.9</v>
       </c>
       <c r="K121">
-        <v>-27.6</v>
+        <v>-34.2</v>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>MSG 1.4x higher at 2050</t>
+          <t>MSG 1.5x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -5984,22 +5984,22 @@
         </is>
       </c>
       <c r="F123">
-        <v>63.67</v>
+        <v>61.91</v>
       </c>
       <c r="G123">
-        <v>73.02</v>
+        <v>65.2</v>
       </c>
       <c r="H123">
-        <v>83.88</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="I123">
-        <v>97.53</v>
+        <v>81.2</v>
       </c>
       <c r="J123">
-        <v>114.79</v>
+        <v>93.02</v>
       </c>
       <c r="K123">
-        <v>136.57</v>
+        <v>108.47</v>
       </c>
     </row>
     <row r="124">
@@ -6029,22 +6029,22 @@
         </is>
       </c>
       <c r="F124">
-        <v>-20.1</v>
+        <v>-21.87</v>
       </c>
       <c r="G124">
-        <v>-12.83</v>
+        <v>-20.64</v>
       </c>
       <c r="H124">
-        <v>-28.55</v>
+        <v>-40.25</v>
       </c>
       <c r="I124">
-        <v>-14.9</v>
+        <v>-31.23</v>
       </c>
       <c r="J124">
-        <v>2.36</v>
+        <v>-19.42</v>
       </c>
       <c r="K124">
-        <v>24.13</v>
+        <v>-3.97</v>
       </c>
     </row>
     <row r="125">
@@ -6074,26 +6074,26 @@
         </is>
       </c>
       <c r="F125">
+        <v>-26.1</v>
+      </c>
+      <c r="G125">
         <v>-24</v>
       </c>
-      <c r="G125">
-        <v>-14.9</v>
-      </c>
       <c r="H125">
-        <v>-25.4</v>
+        <v>-35.8</v>
       </c>
       <c r="I125">
-        <v>-13.3</v>
+        <v>-27.8</v>
       </c>
       <c r="J125">
-        <v>2.1</v>
+        <v>-17.3</v>
       </c>
       <c r="K125">
-        <v>21.5</v>
+        <v>-3.5</v>
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>GCAM 1.2x higher at 2050</t>
+          <t>~4% gap at 2050</t>
         </is>
       </c>
     </row>
@@ -6169,22 +6169,22 @@
         </is>
       </c>
       <c r="F127">
-        <v>143.15</v>
+        <v>143.04</v>
       </c>
       <c r="G127">
-        <v>139.54</v>
+        <v>140.81</v>
       </c>
       <c r="H127">
-        <v>151.98</v>
+        <v>155.02</v>
       </c>
       <c r="I127">
-        <v>154.24</v>
+        <v>156.7</v>
       </c>
       <c r="J127">
-        <v>152.25</v>
+        <v>152.9</v>
       </c>
       <c r="K127">
-        <v>159.13</v>
+        <v>158.99</v>
       </c>
     </row>
     <row r="128">
@@ -6214,22 +6214,22 @@
         </is>
       </c>
       <c r="F128">
-        <v>6.16</v>
+        <v>6.06</v>
       </c>
       <c r="G128">
-        <v>-50.69</v>
+        <v>-49.41</v>
       </c>
       <c r="H128">
-        <v>-40.25</v>
+        <v>-37.21</v>
       </c>
       <c r="I128">
-        <v>-39.97</v>
+        <v>-37.51</v>
       </c>
       <c r="J128">
-        <v>-41.96</v>
+        <v>-41.31</v>
       </c>
       <c r="K128">
-        <v>-35.08</v>
+        <v>-35.22</v>
       </c>
     </row>
     <row r="129">
@@ -6259,19 +6259,19 @@
         </is>
       </c>
       <c r="F129">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="G129">
-        <v>-26.6</v>
+        <v>-26</v>
       </c>
       <c r="H129">
-        <v>-20.9</v>
+        <v>-19.4</v>
       </c>
       <c r="I129">
-        <v>-20.6</v>
+        <v>-19.3</v>
       </c>
       <c r="J129">
-        <v>-21.6</v>
+        <v>-21.3</v>
       </c>
       <c r="K129">
         <v>-18.1</v>
@@ -6354,22 +6354,22 @@
         </is>
       </c>
       <c r="F131">
-        <v>54.65</v>
+        <v>86.77</v>
       </c>
       <c r="G131">
-        <v>194.18</v>
+        <v>250.21</v>
       </c>
       <c r="H131">
-        <v>338.35</v>
+        <v>415.35</v>
       </c>
       <c r="I131">
-        <v>519.6900000000001</v>
+        <v>620.86</v>
       </c>
       <c r="J131">
-        <v>733.0599999999999</v>
+        <v>865.09</v>
       </c>
       <c r="K131">
-        <v>979.33</v>
+        <v>1153.16</v>
       </c>
     </row>
     <row r="132">
@@ -6399,22 +6399,22 @@
         </is>
       </c>
       <c r="F132">
-        <v>-108.39</v>
+        <v>-76.27</v>
       </c>
       <c r="G132">
-        <v>-15.4</v>
+        <v>40.63</v>
       </c>
       <c r="H132">
-        <v>13.41</v>
+        <v>90.42</v>
       </c>
       <c r="I132">
-        <v>27.31</v>
+        <v>128.48</v>
       </c>
       <c r="J132">
-        <v>55.2</v>
+        <v>187.23</v>
       </c>
       <c r="K132">
-        <v>98.38</v>
+        <v>272.2</v>
       </c>
     </row>
     <row r="133">
@@ -6444,26 +6444,26 @@
         </is>
       </c>
       <c r="F133">
-        <v>-66.5</v>
+        <v>-46.8</v>
       </c>
       <c r="G133">
-        <v>-7.3</v>
+        <v>19.4</v>
       </c>
       <c r="H133">
-        <v>4.1</v>
+        <v>27.8</v>
       </c>
       <c r="I133">
-        <v>5.5</v>
+        <v>26.1</v>
       </c>
       <c r="J133">
-        <v>8.1</v>
+        <v>27.6</v>
       </c>
       <c r="K133">
-        <v>11.2</v>
+        <v>30.9</v>
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>GCAM 1.1x higher at 2050</t>
+          <t>GCAM 1.3x higher at 2050</t>
         </is>
       </c>
     </row>
@@ -6539,22 +6539,22 @@
         </is>
       </c>
       <c r="F135">
-        <v>17.42</v>
+        <v>16.41</v>
       </c>
       <c r="G135">
-        <v>42.62</v>
+        <v>32.64</v>
       </c>
       <c r="H135">
-        <v>85.01000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="I135">
-        <v>159.96</v>
+        <v>130.42</v>
       </c>
       <c r="J135">
-        <v>248.4</v>
+        <v>207.6</v>
       </c>
       <c r="K135">
-        <v>342.32</v>
+        <v>286.93</v>
       </c>
     </row>
     <row r="136">
@@ -6584,22 +6584,22 @@
         </is>
       </c>
       <c r="F136">
-        <v>17.42</v>
+        <v>16.41</v>
       </c>
       <c r="G136">
-        <v>42.62</v>
+        <v>32.64</v>
       </c>
       <c r="H136">
-        <v>85.01000000000001</v>
+        <v>65.8</v>
       </c>
       <c r="I136">
-        <v>159.96</v>
+        <v>130.42</v>
       </c>
       <c r="J136">
-        <v>248.4</v>
+        <v>207.6</v>
       </c>
       <c r="K136">
-        <v>342.32</v>
+        <v>286.93</v>
       </c>
     </row>
     <row r="137">
@@ -6630,7 +6630,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>MSG=0, GCAM=342.3</t>
+          <t>MSG=0, GCAM=286.9</t>
         </is>
       </c>
     </row>
@@ -6706,22 +6706,22 @@
         </is>
       </c>
       <c r="F139">
-        <v>1547.56</v>
+        <v>1545.79</v>
       </c>
       <c r="G139">
-        <v>1469.7</v>
+        <v>1468.69</v>
       </c>
       <c r="H139">
-        <v>1427.72</v>
+        <v>1427.81</v>
       </c>
       <c r="I139">
-        <v>1414.12</v>
+        <v>1414.99</v>
       </c>
       <c r="J139">
-        <v>1425.18</v>
+        <v>1426.73</v>
       </c>
       <c r="K139">
-        <v>1463.75</v>
+        <v>1464.71</v>
       </c>
     </row>
     <row r="140">
@@ -6751,22 +6751,22 @@
         </is>
       </c>
       <c r="F140">
-        <v>958.35</v>
+        <v>956.58</v>
       </c>
       <c r="G140">
-        <v>816.62</v>
+        <v>815.61</v>
       </c>
       <c r="H140">
-        <v>774.64</v>
+        <v>774.73</v>
       </c>
       <c r="I140">
-        <v>761.04</v>
+        <v>761.92</v>
       </c>
       <c r="J140">
-        <v>772.1</v>
+        <v>773.65</v>
       </c>
       <c r="K140">
-        <v>810.67</v>
+        <v>811.63</v>
       </c>
     </row>
     <row r="141">
@@ -6796,22 +6796,22 @@
         </is>
       </c>
       <c r="F141">
-        <v>162.7</v>
+        <v>162.4</v>
       </c>
       <c r="G141">
-        <v>125</v>
+        <v>124.9</v>
       </c>
       <c r="H141">
         <v>118.6</v>
       </c>
       <c r="I141">
-        <v>116.5</v>
+        <v>116.7</v>
       </c>
       <c r="J141">
-        <v>118.2</v>
+        <v>118.5</v>
       </c>
       <c r="K141">
-        <v>124.1</v>
+        <v>124.3</v>
       </c>
       <c r="L141" t="inlineStr">
         <is>

</xml_diff>